<commit_message>
brd: Group A doc-accuracy fixes (Pitch Deck Visit Type, Business Registration Task Log)
After per-item verification against the wireframe + Task Dropdowns Master:
- Pitch Deck Log Book: Visit Type corrected to the wireframe's 7 values
  (Site Visit/Phone Call/Pitch Rehearsal/Investor Meeting/Mentoring/Workshop/Other).
- Business Registration Task Log: replaced the generic activity list with the
  12 master tasks.
Verification reclassified the rest (not blind-edited):
- Branding Resources Type: already correct in BRD (audit flag was wrong).
- Logistic 'Implemented' vs 'Completed': BRD standardizes on 'Completed' across
  all 27 frameworks -> standardization decision for BA, not a doc error.
- Task Log column structure (Status/Owner/Due): shared by 5 frameworks ->
  general Log Book normalization (group B).
Matrix data + outputs updated to reflect fixes and reclassifications.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/traceability-matrix.xlsx
+++ b/traceability-matrix.xlsx
@@ -8822,7 +8822,7 @@
       </c>
       <c r="E219" s="2" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F219" s="2" t="inlineStr">
@@ -8832,12 +8832,12 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>BRD DEFECT</t>
+          <t>NOT TESTED</t>
         </is>
       </c>
       <c r="H219" s="2" t="inlineStr">
         <is>
-          <t>BRD lists generic ACTIVITY_TYPES, not the 12 BR_TASKS actually rendered</t>
+          <t>FIXED in BRD: now lists the 12 Task-Master tasks (was a generic activity list)</t>
         </is>
       </c>
     </row>
@@ -9351,7 +9351,7 @@
       </c>
       <c r="H232" s="2" t="inlineStr">
         <is>
-          <t>BRD Task Log shows Status/Owner/Due cols the wireframe lacks; PC_TASKS not enumerated</t>
+          <t>Task-list + column structure (Status/Owner/Due vs wireframe Date/Task/Notes/Attachment) = general Log Book normalization; 5 frameworks share the pattern (see — General row)</t>
         </is>
       </c>
     </row>
@@ -10919,7 +10919,7 @@
       </c>
       <c r="H272" s="2" t="inlineStr">
         <is>
-          <t>BRD says 'Completed' vs wireframe 'Implemented'; omits 'Replace Existing'</t>
+          <t>Standardization decision: BRD uses 'Completed' across all 27 frameworks; logistics wireframes say 'Implemented' — align product or confirm canonical term (BA)</t>
         </is>
       </c>
     </row>
@@ -11345,7 +11345,7 @@
       </c>
       <c r="H283" s="2" t="inlineStr">
         <is>
-          <t>BRD says 'Completed' vs wireframe 'Implemented'</t>
+          <t>Standardization decision: BRD uses 'Completed' across all 27 frameworks; logistics wireframes say 'Implemented' — align product or confirm canonical term (BA)</t>
         </is>
       </c>
     </row>
@@ -13354,7 +13354,7 @@
       </c>
       <c r="E335" s="2" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F335" s="2" t="inlineStr">
@@ -13364,12 +13364,12 @@
       </c>
       <c r="G335" s="2" t="inlineStr">
         <is>
-          <t>BRD DEFECT</t>
+          <t>NOT TESTED</t>
         </is>
       </c>
       <c r="H335" s="2" t="inlineStr">
         <is>
-          <t>Resources Type list missing from BRD</t>
+          <t>Verified present in BRD (Type = Template/Reference/Guideline/Example) — earlier 'missing' flag was incorrect</t>
         </is>
       </c>
     </row>
@@ -14312,7 +14312,7 @@
       </c>
       <c r="E360" s="2" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F360" s="2" t="inlineStr">
@@ -14322,12 +14322,12 @@
       </c>
       <c r="G360" s="2" t="inlineStr">
         <is>
-          <t>BRD DEFECT</t>
+          <t>NOT TESTED</t>
         </is>
       </c>
       <c r="H360" s="2" t="inlineStr">
         <is>
-          <t>BRD lists a DIFFERENT set (Drafting/Review/Mentor Session/Mock Pitch/Investor Meeting) — fix BRD</t>
+          <t>FIXED in BRD: Visit Type now matches the wireframe's 7 values</t>
         </is>
       </c>
     </row>
@@ -18992,7 +18992,7 @@
         <v>0</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
@@ -19312,7 +19312,7 @@
         <v>0</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25">
@@ -19376,7 +19376,7 @@
         <v>1</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="27">
@@ -26708,7 +26708,7 @@
       </c>
       <c r="E186" s="2" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F186" s="2" t="inlineStr">
@@ -26718,12 +26718,12 @@
       </c>
       <c r="G186" s="2" t="inlineStr">
         <is>
-          <t>BRD DEFECT</t>
+          <t>NOT TESTED</t>
         </is>
       </c>
       <c r="H186" s="2" t="inlineStr">
         <is>
-          <t>BRD lists generic ACTIVITY_TYPES, not the 12 BR_TASKS actually rendered</t>
+          <t>FIXED in BRD: now lists the 12 Task-Master tasks (was a generic activity list)</t>
         </is>
       </c>
     </row>
@@ -27199,7 +27199,7 @@
       </c>
       <c r="H198" s="2" t="inlineStr">
         <is>
-          <t>BRD Task Log shows Status/Owner/Due cols the wireframe lacks; PC_TASKS not enumerated</t>
+          <t>Task-list + column structure (Status/Owner/Due vs wireframe Date/Task/Notes/Attachment) = general Log Book normalization; 5 frameworks share the pattern (see — General row)</t>
         </is>
       </c>
     </row>
@@ -28489,7 +28489,7 @@
       </c>
       <c r="H231" s="2" t="inlineStr">
         <is>
-          <t>BRD says 'Completed' vs wireframe 'Implemented'; omits 'Replace Existing'</t>
+          <t>Standardization decision: BRD uses 'Completed' across all 27 frameworks; logistics wireframes say 'Implemented' — align product or confirm canonical term (BA)</t>
         </is>
       </c>
     </row>
@@ -28805,7 +28805,7 @@
       </c>
       <c r="H239" s="2" t="inlineStr">
         <is>
-          <t>BRD says 'Completed' vs wireframe 'Implemented'</t>
+          <t>Standardization decision: BRD uses 'Completed' across all 27 frameworks; logistics wireframes say 'Implemented' — align product or confirm canonical term (BA)</t>
         </is>
       </c>
     </row>
@@ -30312,7 +30312,7 @@
       </c>
       <c r="E278" s="2" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F278" s="2" t="inlineStr">
@@ -30322,12 +30322,12 @@
       </c>
       <c r="G278" s="2" t="inlineStr">
         <is>
-          <t>BRD DEFECT</t>
+          <t>NOT TESTED</t>
         </is>
       </c>
       <c r="H278" s="2" t="inlineStr">
         <is>
-          <t>Resources Type list missing from BRD</t>
+          <t>Verified present in BRD (Type = Template/Reference/Guideline/Example) — earlier 'missing' flag was incorrect</t>
         </is>
       </c>
     </row>
@@ -31156,7 +31156,7 @@
       </c>
       <c r="E300" s="2" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F300" s="2" t="inlineStr">
@@ -31166,12 +31166,12 @@
       </c>
       <c r="G300" s="2" t="inlineStr">
         <is>
-          <t>BRD DEFECT</t>
+          <t>NOT TESTED</t>
         </is>
       </c>
       <c r="H300" s="2" t="inlineStr">
         <is>
-          <t>BRD lists a DIFFERENT set (Drafting/Review/Mentor Session/Mock Pitch/Investor Meeting) — fix BRD</t>
+          <t>FIXED in BRD: Visit Type now matches the wireframe's 7 values</t>
         </is>
       </c>
     </row>
@@ -34702,7 +34702,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -34849,22 +34849,22 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Business Registration</t>
+          <t>Product Compliance</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>dropdown</t>
+          <t>field</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Task Log — 12 BR tasks</t>
+          <t>'Applicable Product' field</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -34879,7 +34879,7 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>BRD lists generic ACTIVITY_TYPES, not the 12 BR_TASKS actually rendered</t>
+          <t>BRD invented this field — NOT in the wireframe</t>
         </is>
       </c>
     </row>
@@ -34896,17 +34896,17 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>field</t>
+          <t>dropdown</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>'Applicable Product' field</t>
+          <t>Task Log — 12 PC tasks</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>P</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -34921,7 +34921,7 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>BRD invented this field — NOT in the wireframe</t>
+          <t>Task-list + column structure (Status/Owner/Due vs wireframe Date/Task/Notes/Attachment) = general Log Book normalization; 5 frameworks share the pattern (see — General row)</t>
         </is>
       </c>
     </row>
@@ -34933,7 +34933,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Product Compliance</t>
+          <t>Logistic Packing</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -34943,7 +34943,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Task Log — 12 PC tasks</t>
+          <t>Impl Status (Intervention &amp; New)</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -34963,7 +34963,7 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>BRD Task Log shows Status/Owner/Due cols the wireframe lacks; PC_TASKS not enumerated</t>
+          <t>Standardization decision: BRD uses 'Completed' across all 27 frameworks; logistics wireframes say 'Implemented' — align product or confirm canonical term (BA)</t>
         </is>
       </c>
     </row>
@@ -34985,7 +34985,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Impl Status (Intervention &amp; New)</t>
+          <t>Resources Category / Log Book Activity Type</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
@@ -35005,7 +35005,7 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>BRD says 'Completed' vs wireframe 'Implemented'; omits 'Replace Existing'</t>
+          <t>BRD Category set differs; Log Book omits several activities</t>
         </is>
       </c>
     </row>
@@ -35017,7 +35017,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Logistic Packing</t>
+          <t>Logistic Service</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -35027,7 +35027,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Resources Category / Log Book Activity Type</t>
+          <t>Implementation Status</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -35047,7 +35047,7 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>BRD Category set differs; Log Book omits several activities</t>
+          <t>Standardization decision: BRD uses 'Completed' across all 27 frameworks; logistics wireframes say 'Implemented' — align product or confirm canonical term (BA)</t>
         </is>
       </c>
     </row>
@@ -35059,7 +35059,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Logistic Service</t>
+          <t>Pitch Deck</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -35069,12 +35069,12 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Implementation Status</t>
+          <t>Task Log Status: Pending/In Progress/Completed/Blocked</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>N</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -35089,29 +35089,29 @@
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>BRD says 'Completed' vs wireframe 'Implemented'</t>
+          <t>'Blocked' option missing from BRD</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Frameworks</t>
+          <t>Entrepreneur Profile</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Branding Identity</t>
+          <t>EP Profile</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>dropdown</t>
+          <t>field</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Resources Category (Brand/Logo/Card/General); Resources Type</t>
+          <t>Rural E Champ Score (Int, permlevel 1 = Core Team only)</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -35121,7 +35121,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -35131,39 +35131,39 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>Resources Type list missing from BRD</t>
+          <t>BRD says 'filled by Fellow'; repo + journey = Core Team only</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Frameworks</t>
+          <t>Entrepreneur Profile</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Pitch Deck</t>
+          <t>EP Profile</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>dropdown</t>
+          <t>field</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Log Book Visit Type (Site/Phone/Pitch Rehearsal/Investor Meeting/Mentoring/Workshop/Other)</t>
+          <t>Status model: activity_status (Active/Inactive) + final_selection (Incubated/Supported); NO stored 'MET'</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -35173,39 +35173,39 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>BRD lists a DIFFERENT set (Drafting/Review/Mentor Session/Mock Pitch/Investor Meeting) — fix BRD</t>
+          <t>BRD/tests treat 'MET' as a stored status; repo has none</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Frameworks</t>
+          <t>Entrepreneur Profile</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Pitch Deck</t>
+          <t>EP Profile</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>dropdown</t>
+          <t>field</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Task Log Status: Pending/In Progress/Completed/Blocked</t>
+          <t>Priority-table 'Applicable?' checkbox</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -35215,7 +35215,7 @@
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>'Blocked' option missing from BRD</t>
+          <t>No 'applicable' field in repo; rows auto-seeded, add/remove hidden — BRD &amp; EP-022 invented it</t>
         </is>
       </c>
     </row>
@@ -35237,7 +35237,7 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Rural E Champ Score (Int, permlevel 1 = Core Team only)</t>
+          <t>Networking: Mentor Master registry doctype</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
@@ -35252,12 +35252,12 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>BRD DEFECT</t>
+          <t>NOT BUILT</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>BRD says 'filled by Fellow'; repo + journey = Core Team only</t>
+          <t>Mentor Master NOT built in repo; PRD specifies it; tests assume it exists</t>
         </is>
       </c>
     </row>
@@ -35274,17 +35274,17 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>field</t>
+          <t>dropdown</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Status model: activity_status (Active/Inactive) + final_selection (Incubated/Supported); NO stored 'MET'</t>
+          <t>Sector: repo = hardcoded 3-option Select</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>P</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
@@ -35298,132 +35298,6 @@
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
-        <is>
-          <t>BRD/tests treat 'MET' as a stored status; repo has none</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>Entrepreneur Profile</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>EP Profile</t>
-        </is>
-      </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>field</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>Priority-table 'Applicable?' checkbox</t>
-        </is>
-      </c>
-      <c r="E15" s="2" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="F15" s="2" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="G15" s="2" t="inlineStr">
-        <is>
-          <t>BRD DEFECT</t>
-        </is>
-      </c>
-      <c r="H15" s="2" t="inlineStr">
-        <is>
-          <t>No 'applicable' field in repo; rows auto-seeded, add/remove hidden — BRD &amp; EP-022 invented it</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>Entrepreneur Profile</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>EP Profile</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>field</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>Networking: Mentor Master registry doctype</t>
-        </is>
-      </c>
-      <c r="E16" s="2" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="F16" s="2" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="G16" s="2" t="inlineStr">
-        <is>
-          <t>NOT BUILT</t>
-        </is>
-      </c>
-      <c r="H16" s="2" t="inlineStr">
-        <is>
-          <t>Mentor Master NOT built in repo; PRD specifies it; tests assume it exists</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>Entrepreneur Profile</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>EP Profile</t>
-        </is>
-      </c>
-      <c r="C17" s="2" t="inlineStr">
-        <is>
-          <t>dropdown</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr">
-        <is>
-          <t>Sector: repo = hardcoded 3-option Select</t>
-        </is>
-      </c>
-      <c r="E17" s="2" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="F17" s="2" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="G17" s="2" t="inlineStr">
-        <is>
-          <t>BRD DEFECT</t>
-        </is>
-      </c>
-      <c r="H17" s="2" t="inlineStr">
         <is>
           <t>journey/BRD/tests assume a Sector master cascading to Business Basket; repo has neither</t>
         </is>

</xml_diff>